<commit_message>
feat(saff-study): publish specification and test suite v1.2
</commit_message>
<xml_diff>
--- a/output/xlsx/CRUDDiagnosticos--GT-.xlsx
+++ b/output/xlsx/CRUDDiagnosticos--GT-.xlsx
@@ -113,16 +113,16 @@
     <t>exibe página com campos de cadastro de novo documento</t>
   </si>
   <si>
-    <t>system: SYSTEM: exibe lista de diagnosticos</t>
-  </si>
-  <si>
-    <t>exibe lista de diagnosticos</t>
-  </si>
-  <si>
-    <t>system: SYSTEM: exibe dados do diagnostico</t>
-  </si>
-  <si>
-    <t>exibe dados do diagnostico</t>
+    <t>system: SYSTEM: exibe lista de diagnósticos</t>
+  </si>
+  <si>
+    <t>exibe lista de diagnósticos</t>
+  </si>
+  <si>
+    <t>system: SYSTEM: exibe dados do diagnóstico</t>
+  </si>
+  <si>
+    <t>exibe dados do diagnóstico</t>
   </si>
   <si>
     <t>system: SYSTEM: retorna a lista de diagnosticos</t>
@@ -149,13 +149,13 @@
     <t>TC3</t>
   </si>
   <si>
-    <t>Alternative Flow 1: Campo fora da formatacao esperada</t>
-  </si>
-  <si>
-    <t>system: SYSTEM: exibe mensagem informando que os dados nao correspondem a formatacao esperada</t>
-  </si>
-  <si>
-    <t>exibe mensagem informando que os dados nao correspondem a formatacao esperada</t>
+    <t>Alternative Flow 1: Campo fora da formatação esperada</t>
+  </si>
+  <si>
+    <t>system: SYSTEM: exibe mensagem informando que os dados nao correspondem a formatação esperada</t>
+  </si>
+  <si>
+    <t>exibe mensagem informando que os dados nao correspondem a formatação esperada</t>
   </si>
   <si>
     <t>TC5</t>
@@ -176,10 +176,10 @@
     <t>Alternative Flow 4: Deleta diagnostico</t>
   </si>
   <si>
-    <t>system: SYSTEM: exibe mensagem solicitando confirmacao</t>
-  </si>
-  <si>
-    <t>exibe mensagem solicitando confirmacao</t>
+    <t>system: SYSTEM: exibe mensagem solicitando confirmaçao</t>
+  </si>
+  <si>
+    <t>exibe mensagem solicitando confirmaçao</t>
   </si>
   <si>
     <t>TC7</t>

</xml_diff>